<commit_message>
commit right config and exp files
</commit_message>
<xml_diff>
--- a/docs/vs/VSTableFreehand/VSTable.xlsx
+++ b/docs/vs/VSTableFreehand/VSTable.xlsx
@@ -9,13 +9,12 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="7455" yWindow="1305" windowWidth="23550" windowHeight="13290" activeTab="2"/>
+    <workbookView xWindow="7455" yWindow="1305" windowWidth="13035" windowHeight="6840" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="OverView" sheetId="5" r:id="rId1"/>
     <sheet name="Table" sheetId="2" r:id="rId2"/>
-    <sheet name="EMTable" sheetId="3" r:id="rId3"/>
-    <sheet name="FormTable" sheetId="4" r:id="rId4"/>
+    <sheet name="embedded FormTable" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="138">
   <si>
     <r>
       <t xml:space="preserve">1.  Binding </t>
@@ -706,8 +705,128 @@
     <t>AutoCase: Table_Case.groovy/NT7</t>
   </si>
   <si>
-    <r>
-      <t>2. worksheet</t>
+    <t>1. one value or multi value on  null, date,time,other</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2. data path: header, detail</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Note: copy Highlight manual check</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Table</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Testing</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">use partly col and set col </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>visisble</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. use datetime, time, date col type</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2. use form to change cell value and store to bk</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. use form to change cell value</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VS:Table/EFT2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AutoCase: Table_Case.groovy/EFT2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3.add/modify/delete rows</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>delete row and header in embedded form table</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>add and modify in embedded form table</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>integer/text/date/boolean/combobox input</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>delete row(first,middle,last) and table header</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>add(first,middle,last) and modify rows</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>auto case</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>check</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>un-submitted changes</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>highlight and condition</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FormImport:</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FormTable_Case.groovy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+      </rPr>
+      <t>覆盖</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>column options</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>4.condition, highlight</t>
     </r>
     <r>
       <rPr>
@@ -717,64 +836,115 @@
         <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t>中embdded table的属性对vs中table的影响</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">    1) max row </t>
-    </r>
-    <r>
-      <rPr>
+      <t>等要正式提交之后才应用</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>//</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="宋体"/>
         <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t>在vs中不应用</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>VS Embedded table</t>
-    </r>
-    <r>
-      <rPr>
+      <t>删除</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>table header, date/time</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="宋体"/>
         <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t>中没有应用</t>
-    </r>
-    <r>
-      <rPr>
+      <t>的</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>,</t>
-    </r>
-    <r>
-      <rPr>
+      <t>format</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
         <sz val="10"/>
         <color theme="1"/>
         <rFont val="宋体"/>
         <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t>但是移动scroll之后, 会显示limit的信息, 不对??</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">     1) </t>
+      <t>不对，</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>ignore</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+      </rPr>
+      <t>覆盖</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>embedded form table</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+      </rPr>
+      <t/>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>5.Write-Back</t>
     </r>
     <r>
       <rPr>
@@ -784,311 +954,12 @@
         <family val="3"/>
         <charset val="134"/>
       </rPr>
-      <t>双击编辑</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">     2) form </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>组件控制</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">     3) Script</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">3. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>对Cell value进行编辑, 对其他数据的影响, 结合Write-Back的应用</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1. only binding ws embdded table</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>//manual check</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1. one value or multi value on  null, date,time,other</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2. data path: header, detail</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Note: copy Highlight manual check</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1. Table</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Testing</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">use partly col and set col </t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>visisble</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1. use datetime, time, date col type</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2. use form to change cell value and store to bk</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1. use form to change cell value</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>VS:Table/EFT2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AutoCase: Table_Case.groovy/EFT2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>3.add/modify/delete rows</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>delete row and header in embedded form table</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>add and modify in embedded form table</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>integer/text/date/boolean/combobox input</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>delete row(first,middle,last) and table header</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>add(first,middle,last) and modify rows</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>add delete and modify rows</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>float/combobox(embedded+query) input</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>add/delete/modify rows</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>auto case</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>check</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>un-submitted changes</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>highlight and condition</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>FormImport:</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>FormTable_Case.groovy</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>1.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-      </rPr>
-      <t>覆盖</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>embedded table+form table</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-      </rPr>
-      <t>和普通</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>form table</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>2.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="2"/>
-      </rPr>
-      <t>覆盖</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>column options</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>4.condition, highlight</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>等要正式提交之后才应用</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>//</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>删除</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>table header, date/time</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>的</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>format</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>不对，</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>ignore</t>
-    </r>
+      <t>的应用</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>change cell value by form component</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1153,7 +1024,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1169,12 +1040,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1323,7 +1188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1348,7 +1213,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1941,12 +1805,12 @@
         <v>37</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C37" s="2" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.2">
@@ -1954,7 +1818,7 @@
         <v>38</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.2">
@@ -1964,7 +1828,7 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.2">
@@ -2392,287 +2256,205 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:N18"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="5.125" style="2" customWidth="1"/>
-    <col min="2" max="16384" width="9" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B3" s="2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B4" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B5" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G5" s="20" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B7" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B8" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B9" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B10" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A13" s="5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B15" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="17"/>
-      <c r="I15" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="J15" s="16"/>
-      <c r="K15" s="16"/>
-      <c r="L15" s="17"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B16" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J16" s="12"/>
-      <c r="K16" s="12"/>
-      <c r="L16" s="7"/>
-      <c r="N16" s="19" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B17" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="9"/>
-      <c r="N17" s="18" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B18" s="10"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="14"/>
-      <c r="L18" s="11"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B2" s="5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="C3" s="2" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="C4" s="2" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="C5" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="C6" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C7" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B8" s="5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B9" s="5"/>
       <c r="C9" s="15" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="17"/>
       <c r="G9" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="23"/>
-      <c r="K9" s="24" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+        <v>127</v>
+      </c>
+      <c r="H9" s="21"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="23" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="C10" s="6" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="D10" s="12"/>
       <c r="E10" s="12"/>
       <c r="F10" s="7"/>
       <c r="G10" s="6" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
       <c r="J10" s="7"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="C11" s="10"/>
       <c r="D11" s="14"/>
       <c r="E11" s="14"/>
       <c r="F11" s="11"/>
       <c r="G11" s="10" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
       <c r="J11" s="11"/>
-      <c r="K11" s="24" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="C12" s="21" t="s">
-        <v>131</v>
-      </c>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="21" t="s">
+      <c r="K11" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="H12" s="22"/>
-      <c r="I12" s="22"/>
-      <c r="J12" s="23"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="C13" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="7"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="C14" s="10"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="10" t="s">
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C12" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="H12" s="21"/>
+      <c r="I12" s="21"/>
+      <c r="J12" s="22"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C13" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="H13" s="21"/>
+      <c r="I13" s="21"/>
+      <c r="J13" s="22"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C15" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="H14" s="14"/>
-      <c r="I14" s="14"/>
-      <c r="J14" s="11"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="C15" s="21" t="s">
-        <v>140</v>
-      </c>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="23"/>
-      <c r="G15" s="21" t="s">
-        <v>141</v>
-      </c>
-      <c r="H15" s="22"/>
-      <c r="I15" s="22"/>
-      <c r="J15" s="23"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C16" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" s="17"/>
+      <c r="E16" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="17"/>
+    </row>
+    <row r="17" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="C17" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D17" s="7"/>
+      <c r="E17" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="7"/>
+      <c r="O17" s="19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="18" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="C18" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="D18" s="9"/>
+      <c r="E18" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="13"/>
+      <c r="M18" s="9"/>
+      <c r="O18" s="18" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="19" spans="3:15" x14ac:dyDescent="0.2">
+      <c r="C19" s="10"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="14"/>
+      <c r="L19" s="14"/>
+      <c r="M19" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>